<commit_message>
mantenimiento en el script, ademas de añadido try catch para capturar errores, y añadido un formateo al grado por si solo se ingresa un numero -> 4 -> 4°
</commit_message>
<xml_diff>
--- a/Planillas/Listado_Alumnos.xlsx
+++ b/Planillas/Listado_Alumnos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0dd53fed1783efb5/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0dd53fed1783efb5/Escritorio/Fátima 2026/generador-certificados/Planillas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="409" documentId="8_{9578C5D7-98C8-4D67-8E48-62822BB58908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B3A2BD1-EB83-488C-BF9C-1932872561D8}"/>
+  <xr:revisionPtr revIDLastSave="411" documentId="8_{9578C5D7-98C8-4D67-8E48-62822BB58908}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF3753C7-EE65-4F52-95D9-2B32BC8485C6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{7EDD2DAE-180A-4C76-8E2D-2347D9F69EAE}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>localidad</t>
   </si>
@@ -72,72 +72,6 @@
   </si>
   <si>
     <t>apellido</t>
-  </si>
-  <si>
-    <t>rodriguez</t>
-  </si>
-  <si>
-    <t>christian</t>
-  </si>
-  <si>
-    <t>2°</t>
-  </si>
-  <si>
-    <t>Marcos fernando rodriguez</t>
-  </si>
-  <si>
-    <t>La policia de salta y la policia de la provincia de santa cruz de la argentina</t>
-  </si>
-  <si>
-    <t>rio gallegos</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
-    <t>Alvarez</t>
-  </si>
-  <si>
-    <t>marilu</t>
-  </si>
-  <si>
-    <t>5°</t>
-  </si>
-  <si>
-    <t>padre</t>
-  </si>
-  <si>
-    <t>madre</t>
-  </si>
-  <si>
-    <t>maria alvarez</t>
-  </si>
-  <si>
-    <t>correo argentino</t>
-  </si>
-  <si>
-    <t>salta</t>
-  </si>
-  <si>
-    <t>f</t>
-  </si>
-  <si>
-    <t>dsadsa</t>
-  </si>
-  <si>
-    <t>dasdsadas</t>
-  </si>
-  <si>
-    <t>tutor</t>
-  </si>
-  <si>
-    <t>hospital</t>
-  </si>
-  <si>
-    <t>dsd</t>
-  </si>
-  <si>
-    <t>fgfdgfdgdf</t>
   </si>
 </sst>
 </file>
@@ -236,10 +170,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -612,126 +542,50 @@
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A2" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="4">
-        <v>89654123</v>
-      </c>
-      <c r="D2" s="2">
-        <v>35499</v>
-      </c>
-      <c r="E2" s="3">
-        <v>29</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="4">
-        <v>21318758</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>18</v>
-      </c>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="4">
-        <v>38456963</v>
-      </c>
-      <c r="D3" s="2">
-        <v>33965</v>
-      </c>
-      <c r="E3" s="3">
-        <v>33</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="4">
-        <v>87456321</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C4" s="4">
-        <v>38456963</v>
-      </c>
-      <c r="D4" s="2">
-        <v>33966</v>
-      </c>
-      <c r="E4" s="3">
-        <v>33</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I4" s="4">
-        <v>87456321</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="4"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="4"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="A5" s="3"/>
+      <c r="B5" s="3"/>
       <c r="C5" s="4"/>
       <c r="D5" s="2"/>
       <c r="E5" s="3"/>

</xml_diff>